<commit_message>
Sync planning SharePoint : S26
</commit_message>
<xml_diff>
--- a/Plannings 2026 S26.xlsx
+++ b/Plannings 2026 S26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A23AA2D1-9819-4B65-9C3A-D83FC30F8B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{A23AA2D1-9819-4B65-9C3A-D83FC30F8B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE77D127-EEBA-4B11-B64D-E4268FA37DEA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="151">
   <si>
     <t>Planning des salariés du 22/06/2026 au 28/06/2026</t>
   </si>
@@ -126,9 +126,6 @@
     <t>11:45/15:00</t>
   </si>
   <si>
-    <t>10:30/17:00</t>
-  </si>
-  <si>
     <t>COMMD</t>
   </si>
   <si>
@@ -450,9 +447,6 @@
     <t>18:30/23:30</t>
   </si>
   <si>
-    <t>11:50/17:00</t>
-  </si>
-  <si>
     <t>Commercial : EDF et BetssonLeagues</t>
   </si>
   <si>
@@ -472,6 +466,15 @@
   </si>
   <si>
     <t>EDF // ANNIV // FINALES LEAGUES</t>
+  </si>
+  <si>
+    <t>10:00/17:00</t>
+  </si>
+  <si>
+    <t>11:25/18:30</t>
+  </si>
+  <si>
+    <t>10:15/17:00</t>
   </si>
 </sst>
 </file>
@@ -985,7 +988,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1021,6 +1024,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1206,6 +1212,12 @@
     <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5270,6 +5282,314 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2241176" y="2723029"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="103" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C7669B8-BCA5-4733-81DE-47FB25117A0D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="4391025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="104" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77D8CB80-1702-4EE3-9D7B-BDF49E049259}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1219200" y="4391025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="105" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6347A111-1ED8-4B80-836E-D5F3B3359280}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="4391025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="106" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B2FD599-492F-45B5-B893-DEA300AB543A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="4772025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="107" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F23C95C-35F8-412F-8468-1A1B3CE82A77}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="5153025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="108" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{937BD91D-3F12-47A4-9079-ABF15B051E30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="4391025"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="109" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{931ABFC2-BA31-46B2-84CF-FFE1562B4443}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3657600" y="4391025"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5680,162 +6000,162 @@
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="65" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="67"/>
+    </row>
+    <row r="4" spans="1:8" s="68" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B4" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="69" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="66"/>
-    </row>
-    <row r="4" spans="1:8" s="67" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B4" s="68" t="s">
+      <c r="D4" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="C4" s="68" t="s">
+      <c r="E4" s="69" t="s">
         <v>145</v>
       </c>
-      <c r="D4" s="68" t="s">
+      <c r="F4" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="E4" s="68" t="s">
+      <c r="G4" s="69" t="s">
         <v>147</v>
       </c>
-      <c r="F4" s="68" t="s">
-        <v>148</v>
-      </c>
-      <c r="G4" s="68" t="s">
-        <v>149</v>
-      </c>
-      <c r="H4" s="68" t="s">
-        <v>76</v>
+      <c r="H4" s="69" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="54" t="s">
+      <c r="B6" s="18"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="20"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="57" t="s">
+      <c r="A7" s="21"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="41" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="20"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="20"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="42" t="s">
+      <c r="A9" s="21"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="24"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="18"/>
-      <c r="H10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="20"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="24"/>
+      <c r="A11" s="25"/>
       <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="60" t="s">
+      <c r="D11" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="E11" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="58" t="s">
-        <v>138</v>
+      <c r="F11" s="59" t="s">
+        <v>137</v>
       </c>
       <c r="G11" s="1"/>
-      <c r="H11" s="25"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="24"/>
-      <c r="B12" s="59" t="s">
+      <c r="A12" s="25"/>
+      <c r="B12" s="60" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="1"/>
@@ -5847,11 +6167,11 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="25"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="24"/>
-      <c r="B13" s="60" t="s">
+      <c r="A13" s="25"/>
+      <c r="B13" s="61" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="1"/>
@@ -5863,451 +6183,447 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="25"/>
+      <c r="H13" s="26"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="24"/>
-      <c r="B14" s="60"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="61"/>
       <c r="C14" s="1"/>
-      <c r="D14" s="44" t="s">
+      <c r="D14" s="45" t="s">
         <v>20</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="25"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="20"/>
-      <c r="B15" s="61"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="42" t="s">
+      <c r="A15" s="21"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="24"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="30"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="59"/>
+      <c r="F17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="G17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="H17" s="59"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="59" t="s">
+        <v>138</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="59" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59" t="s">
+        <v>149</v>
+      </c>
+      <c r="G18" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="H18" s="59"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="13"/>
+      <c r="B19" s="59"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="75" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="59"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="59"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="13"/>
+      <c r="B20" s="59"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="76" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="59"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="13"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="19"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="58" t="s">
-        <v>139</v>
-      </c>
-      <c r="C18" s="58" t="s">
-        <v>142</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="58" t="s">
-        <v>139</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H18" s="25"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="24"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="59" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="25"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="24"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="60" t="s">
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+      <c r="H21" s="59"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="13"/>
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="25"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="24"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="25"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22" t="s">
+      <c r="E22" s="59"/>
+      <c r="F22" s="59"/>
+      <c r="G22" s="59"/>
+      <c r="H22" s="59"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="23"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="37" t="s">
+      <c r="B23" s="39"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="41"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="40"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="B24" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="C24" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="F24" s="41" t="s">
+      <c r="G24" s="19"/>
+      <c r="H24" s="20"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="25"/>
+      <c r="B25" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="19"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="24"/>
-      <c r="B25" s="55" t="s">
+      <c r="C25" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="56" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="55" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="55" t="s">
+      <c r="E25" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="55" t="s">
+      <c r="F25" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="F25" s="43" t="s">
+      <c r="G25" s="1"/>
+      <c r="H25" s="26"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="25"/>
+      <c r="B26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G25" s="1"/>
-      <c r="H25" s="25"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="24"/>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="56" t="s">
-        <v>40</v>
+      <c r="D26" s="57" t="s">
+        <v>39</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="43"/>
+      <c r="F26" s="44"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="25"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="24"/>
+      <c r="A27" s="25"/>
       <c r="B27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="D27" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="D27" s="55" t="s">
+      <c r="E27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="44"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="26"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="25"/>
+      <c r="B28" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="1"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="26"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="25"/>
+      <c r="B29" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="F27" s="43"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="25"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="24"/>
-      <c r="B28" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="25"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="24"/>
-      <c r="B29" s="55" t="s">
+      <c r="C29" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="55" t="s">
+      <c r="D29" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="E29" s="1"/>
-      <c r="F29" s="43"/>
+      <c r="F29" s="44"/>
       <c r="G29" s="1"/>
-      <c r="H29" s="25"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="24"/>
-      <c r="B30" s="55"/>
+      <c r="A30" s="25"/>
+      <c r="B30" s="56"/>
       <c r="C30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="56" t="s">
-        <v>40</v>
+      <c r="D30" s="57" t="s">
+        <v>39</v>
       </c>
       <c r="E30" s="1"/>
-      <c r="F30" s="43"/>
+      <c r="F30" s="44"/>
       <c r="G30" s="1"/>
-      <c r="H30" s="25"/>
+      <c r="H30" s="26"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="20"/>
-      <c r="B31" s="57"/>
-      <c r="C31" s="22" t="s">
+      <c r="A31" s="21"/>
+      <c r="B31" s="58"/>
+      <c r="C31" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="57" t="s">
+      <c r="E31" s="23"/>
+      <c r="F31" s="43"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="24"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="22"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="23"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="H32" s="20"/>
+    </row>
+    <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="21"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="58" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="24"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="54" t="s">
-        <v>12</v>
-      </c>
-      <c r="H32" s="19"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="20"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="23"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+      <c r="B34" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="D34" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="E34" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="54" t="s">
+      <c r="F34" s="19"/>
+      <c r="G34" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="25"/>
+      <c r="B35" s="59" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="24"/>
-      <c r="B35" s="58" t="s">
-        <v>140</v>
-      </c>
-      <c r="C35" s="46" t="s">
+      <c r="D35" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="D35" s="55" t="s">
+      <c r="E35" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H35" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="H35" s="25" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="24"/>
+      <c r="A36" s="25"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="46"/>
+      <c r="C36" s="47"/>
       <c r="D36" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="44" t="s">
+      <c r="E36" s="45" t="s">
         <v>15</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="44" t="s">
+      <c r="G36" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="H36" s="25"/>
+      <c r="H36" s="26"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="24"/>
+      <c r="A37" s="25"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="46"/>
+      <c r="C37" s="47"/>
       <c r="D37" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E37" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="E37" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="H37" s="25"/>
+      <c r="H37" s="26"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="24"/>
+      <c r="A38" s="25"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="43"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="57" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" s="44"/>
       <c r="F38" s="1"/>
       <c r="G38" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="25"/>
+      <c r="H38" s="26"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="24"/>
+      <c r="A39" s="25"/>
       <c r="B39" s="1"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="55" t="s">
-        <v>68</v>
-      </c>
-      <c r="E39" s="43"/>
+      <c r="C39" s="47"/>
+      <c r="D39" s="56" t="s">
+        <v>67</v>
+      </c>
+      <c r="E39" s="44"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H39" s="25"/>
+      <c r="H39" s="26"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="24"/>
+      <c r="A40" s="25"/>
       <c r="B40" s="1"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="44" t="s">
+      <c r="C40" s="47"/>
+      <c r="D40" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="E40" s="44"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="E40" s="43"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="45" t="s">
+      <c r="H40" s="26"/>
+    </row>
+    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="21"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="H40" s="25"/>
-    </row>
-    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="20"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="42" t="s">
+      <c r="E41" s="43"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="E41" s="42"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="47" t="s">
+      <c r="H41" s="24"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="33" t="s">
         <v>72</v>
-      </c>
-      <c r="H41" s="23"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
-        <v>73</v>
       </c>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -6317,232 +6633,232 @@
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
-      <c r="H42" s="25"/>
+      <c r="H42" s="26"/>
     </row>
     <row r="43" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="20"/>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="23"/>
+      <c r="A43" s="21"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="F43" s="23"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
+      <c r="A44" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="B44" s="49" t="s">
-        <v>136</v>
-      </c>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="E44" s="18"/>
-      <c r="F44" s="18"/>
-      <c r="G44" s="51" t="s">
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="H44" s="20"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="25"/>
+      <c r="B45" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="H44" s="19"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="24"/>
-      <c r="B45" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-      <c r="G45" s="52" t="s">
-        <v>79</v>
-      </c>
-      <c r="H45" s="25"/>
+      <c r="G45" s="53" t="s">
+        <v>78</v>
+      </c>
+      <c r="H45" s="26"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="24"/>
-      <c r="B46" s="50" t="s">
-        <v>137</v>
+      <c r="A46" s="25"/>
+      <c r="B46" s="51" t="s">
+        <v>136</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
-      <c r="G46" s="52"/>
-      <c r="H46" s="25"/>
+      <c r="G46" s="53"/>
+      <c r="H46" s="26"/>
     </row>
     <row r="47" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="20"/>
-      <c r="B47" s="22" t="s">
+      <c r="A47" s="21"/>
+      <c r="B47" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="24"/>
+    </row>
+    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="53"/>
-      <c r="H47" s="23"/>
-    </row>
-    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+      <c r="B48" s="28"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="30"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="B48" s="27"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="28"/>
-      <c r="H48" s="29"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
+      <c r="B49" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G49" s="19"/>
+      <c r="H49" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="21"/>
+      <c r="B50" s="64" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="G50" s="23"/>
+      <c r="H50" s="24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="70" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="21"/>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="71" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B53" s="35"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="36"/>
+      <c r="E53" s="36"/>
+      <c r="F53" s="36"/>
+      <c r="G53" s="36"/>
+      <c r="H53" s="37"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B54" s="19"/>
+      <c r="C54" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="D54" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="H54" s="20"/>
+    </row>
+    <row r="55" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="21"/>
+      <c r="B55" s="23"/>
+      <c r="C55" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="D55" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="H55" s="24"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" s="19"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="H56" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C49" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="D49" s="18"/>
-      <c r="E49" s="18"/>
-      <c r="F49" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G49" s="18"/>
-      <c r="H49" s="19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="20"/>
-      <c r="B50" s="63" t="s">
-        <v>141</v>
-      </c>
-      <c r="C50" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="G50" s="22"/>
-      <c r="H50" s="23" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="B51" s="18"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="18"/>
-      <c r="H51" s="69" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="20"/>
-      <c r="B52" s="22"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="70" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="B53" s="34"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="35"/>
-      <c r="F53" s="35"/>
-      <c r="G53" s="35"/>
-      <c r="H53" s="36"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B54" s="18"/>
-      <c r="C54" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="D54" s="41" t="s">
-        <v>69</v>
-      </c>
-      <c r="E54" s="18"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="H54" s="19"/>
-    </row>
-    <row r="55" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="20"/>
-      <c r="B55" s="22"/>
-      <c r="C55" s="47" t="s">
-        <v>61</v>
-      </c>
-      <c r="D55" s="42" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="47" t="s">
-        <v>88</v>
-      </c>
-      <c r="H55" s="23"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B56" s="18"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="18"/>
-      <c r="E56" s="18"/>
-      <c r="F56" s="18"/>
-      <c r="G56" s="51" t="s">
-        <v>76</v>
-      </c>
-      <c r="H56" s="19" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="24"/>
+      <c r="A57" s="25"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
-      <c r="G57" s="52" t="s">
+      <c r="G57" s="53" t="s">
+        <v>89</v>
+      </c>
+      <c r="H57" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="H57" s="25" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="24"/>
+      <c r="A58" s="25"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
@@ -6551,151 +6867,151 @@
       <c r="G58" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H58" s="71" t="s">
-        <v>76</v>
+      <c r="H58" s="72" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="24"/>
+      <c r="A59" s="25"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
       <c r="G59" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H59" s="73" t="s">
         <v>92</v>
       </c>
-      <c r="H59" s="72" t="s">
-        <v>93</v>
-      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="24"/>
+      <c r="A60" s="25"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
-      <c r="H60" s="31" t="s">
+      <c r="H60" s="32" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="24"/>
+      <c r="A61" s="25"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
-      <c r="H61" s="25" t="s">
-        <v>94</v>
+      <c r="H61" s="26" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="24"/>
+      <c r="A62" s="25"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
-      <c r="H62" s="31" t="s">
+      <c r="H62" s="32" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="24"/>
+      <c r="A63" s="25"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
-      <c r="H63" s="25" t="s">
-        <v>95</v>
+      <c r="H63" s="26" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="24"/>
+      <c r="A64" s="25"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
-      <c r="H64" s="71" t="s">
-        <v>76</v>
+      <c r="H64" s="72" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="20"/>
-      <c r="B65" s="22"/>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="22"/>
-      <c r="G65" s="22"/>
-      <c r="H65" s="70" t="s">
-        <v>90</v>
+      <c r="A65" s="21"/>
+      <c r="B65" s="23"/>
+      <c r="C65" s="23"/>
+      <c r="D65" s="23"/>
+      <c r="E65" s="23"/>
+      <c r="F65" s="23"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="71" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="16" t="s">
+      <c r="A66" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="E66" s="19"/>
+      <c r="F66" s="19"/>
+      <c r="G66" s="19"/>
+      <c r="H66" s="20"/>
+    </row>
+    <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="21"/>
+      <c r="B67" s="23"/>
+      <c r="C67" s="23"/>
+      <c r="D67" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="E67" s="23"/>
+      <c r="F67" s="23"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="24"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="B66" s="18"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="41" t="s">
-        <v>69</v>
-      </c>
-      <c r="E66" s="18"/>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
-      <c r="H66" s="19"/>
-    </row>
-    <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="20"/>
-      <c r="B67" s="22"/>
-      <c r="C67" s="22"/>
-      <c r="D67" s="42" t="s">
-        <v>71</v>
-      </c>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="23"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" s="16" t="s">
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="19"/>
+      <c r="F68" s="19"/>
+      <c r="G68" s="19"/>
+      <c r="H68" s="70" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="21"/>
+      <c r="B69" s="23"/>
+      <c r="C69" s="23"/>
+      <c r="D69" s="23"/>
+      <c r="E69" s="23"/>
+      <c r="F69" s="23"/>
+      <c r="G69" s="23"/>
+      <c r="H69" s="71" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="33" t="s">
         <v>97</v>
-      </c>
-      <c r="B68" s="18"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="18"/>
-      <c r="E68" s="18"/>
-      <c r="F68" s="18"/>
-      <c r="G68" s="18"/>
-      <c r="H68" s="69" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="20"/>
-      <c r="B69" s="22"/>
-      <c r="C69" s="22"/>
-      <c r="D69" s="22"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="70" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="32" t="s">
-        <v>98</v>
       </c>
       <c r="B70" s="1"/>
       <c r="C70" s="1" t="s">
@@ -6711,28 +7027,28 @@
         <v>18</v>
       </c>
       <c r="G70" s="1"/>
-      <c r="H70" s="25"/>
+      <c r="H70" s="26"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" s="24"/>
+      <c r="A71" s="25"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="F71" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F71" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="G71" s="1"/>
-      <c r="H71" s="25"/>
+      <c r="H71" s="26"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" s="24"/>
+      <c r="A72" s="25"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="2" t="s">
@@ -6741,240 +7057,240 @@
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
-      <c r="H72" s="25"/>
+      <c r="H72" s="26"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" s="24"/>
+      <c r="A73" s="25"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
       <c r="D73" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
-      <c r="H73" s="25"/>
+      <c r="H73" s="26"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="24"/>
+      <c r="A74" s="25"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
-      <c r="D74" s="44" t="s">
+      <c r="D74" s="45" t="s">
         <v>15</v>
       </c>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
-      <c r="H74" s="25"/>
+      <c r="H74" s="26"/>
     </row>
     <row r="75" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="20"/>
-      <c r="B75" s="22"/>
-      <c r="C75" s="22"/>
-      <c r="D75" s="42" t="s">
+      <c r="A75" s="21"/>
+      <c r="B75" s="23"/>
+      <c r="C75" s="23"/>
+      <c r="D75" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="E75" s="23"/>
+      <c r="F75" s="23"/>
+      <c r="G75" s="23"/>
+      <c r="H75" s="24"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="22"/>
-      <c r="H75" s="23"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B76" s="18"/>
-      <c r="C76" s="18"/>
-      <c r="D76" s="18"/>
-      <c r="E76" s="18"/>
-      <c r="F76" s="18"/>
-      <c r="G76" s="51" t="s">
-        <v>76</v>
-      </c>
-      <c r="H76" s="69" t="s">
-        <v>76</v>
+      <c r="B76" s="19"/>
+      <c r="C76" s="19"/>
+      <c r="D76" s="19"/>
+      <c r="E76" s="19"/>
+      <c r="F76" s="19"/>
+      <c r="G76" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="H76" s="70" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A77" s="24"/>
+      <c r="A77" s="25"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
-      <c r="G77" s="52" t="s">
+      <c r="G77" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="H77" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="H77" s="72" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A78" s="24"/>
+      <c r="A78" s="25"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
-      <c r="G78" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="H78" s="71" t="s">
-        <v>76</v>
+      <c r="G78" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="H78" s="72" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" s="24"/>
+      <c r="A79" s="25"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
-      <c r="G79" s="46" t="s">
-        <v>88</v>
-      </c>
-      <c r="H79" s="72" t="s">
-        <v>108</v>
+      <c r="G79" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="H79" s="73" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A80" s="24"/>
+      <c r="A80" s="25"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
-      <c r="G80" s="46"/>
-      <c r="H80" s="71" t="s">
-        <v>109</v>
+      <c r="G80" s="47"/>
+      <c r="H80" s="72" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A81" s="24"/>
+      <c r="A81" s="25"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
-      <c r="G81" s="46"/>
-      <c r="H81" s="72" t="s">
-        <v>110</v>
+      <c r="G81" s="47"/>
+      <c r="H81" s="73" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A82" s="24"/>
+      <c r="A82" s="25"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
-      <c r="G82" s="46"/>
-      <c r="H82" s="31" t="s">
+      <c r="G82" s="47"/>
+      <c r="H82" s="32" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="20"/>
-      <c r="B83" s="22"/>
-      <c r="C83" s="22"/>
-      <c r="D83" s="22"/>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="47"/>
-      <c r="H83" s="23" t="s">
+      <c r="A83" s="21"/>
+      <c r="B83" s="23"/>
+      <c r="C83" s="23"/>
+      <c r="D83" s="23"/>
+      <c r="E83" s="23"/>
+      <c r="F83" s="23"/>
+      <c r="G83" s="48"/>
+      <c r="H83" s="24" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="27" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="26" t="s">
+      <c r="B84" s="28"/>
+      <c r="C84" s="29"/>
+      <c r="D84" s="29"/>
+      <c r="E84" s="29"/>
+      <c r="F84" s="29"/>
+      <c r="G84" s="29"/>
+      <c r="H84" s="30"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="B84" s="27"/>
-      <c r="C84" s="28"/>
-      <c r="D84" s="28"/>
-      <c r="E84" s="28"/>
-      <c r="F84" s="28"/>
-      <c r="G84" s="28"/>
-      <c r="H84" s="29"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A85" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="B85" s="18"/>
-      <c r="C85" s="18"/>
-      <c r="D85" s="18"/>
-      <c r="E85" s="18"/>
-      <c r="F85" s="18"/>
-      <c r="G85" s="54" t="s">
+      <c r="B85" s="19"/>
+      <c r="C85" s="19"/>
+      <c r="D85" s="19"/>
+      <c r="E85" s="19"/>
+      <c r="F85" s="19"/>
+      <c r="G85" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="H85" s="19"/>
+      <c r="H85" s="20"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A86" s="24"/>
+      <c r="A86" s="25"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
-      <c r="G86" s="55" t="s">
+      <c r="G86" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="H86" s="25"/>
+      <c r="H86" s="26"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A87" s="24"/>
+      <c r="A87" s="25"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
       <c r="D87" s="1"/>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
-      <c r="G87" s="56" t="s">
+      <c r="G87" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="H87" s="25"/>
+      <c r="H87" s="26"/>
     </row>
     <row r="88" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="20"/>
-      <c r="B88" s="22"/>
-      <c r="C88" s="22"/>
-      <c r="D88" s="22"/>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
-      <c r="G88" s="57" t="s">
-        <v>42</v>
-      </c>
-      <c r="H88" s="23"/>
+      <c r="A88" s="21"/>
+      <c r="B88" s="23"/>
+      <c r="C88" s="23"/>
+      <c r="D88" s="23"/>
+      <c r="E88" s="23"/>
+      <c r="F88" s="23"/>
+      <c r="G88" s="58" t="s">
+        <v>41</v>
+      </c>
+      <c r="H88" s="24"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A89" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B89" s="18"/>
-      <c r="C89" s="18"/>
-      <c r="D89" s="18"/>
-      <c r="E89" s="18"/>
-      <c r="F89" s="18"/>
-      <c r="G89" s="51" t="s">
-        <v>76</v>
-      </c>
-      <c r="H89" s="19"/>
+      <c r="A89" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B89" s="19"/>
+      <c r="C89" s="19"/>
+      <c r="D89" s="19"/>
+      <c r="E89" s="19"/>
+      <c r="F89" s="19"/>
+      <c r="G89" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="H89" s="20"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A90" s="24"/>
+      <c r="A90" s="25"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
-      <c r="G90" s="52" t="s">
+      <c r="G90" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="H90" s="25"/>
+      <c r="H90" s="26"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A91" s="24"/>
+      <c r="A91" s="25"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
       <c r="D91" s="1"/>
@@ -6983,48 +7299,48 @@
       <c r="G91" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H91" s="25"/>
+      <c r="H91" s="26"/>
     </row>
     <row r="92" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="20"/>
-      <c r="B92" s="22"/>
-      <c r="C92" s="22"/>
-      <c r="D92" s="22"/>
-      <c r="E92" s="22"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="22" t="s">
+      <c r="A92" s="21"/>
+      <c r="B92" s="23"/>
+      <c r="C92" s="23"/>
+      <c r="D92" s="23"/>
+      <c r="E92" s="23"/>
+      <c r="F92" s="23"/>
+      <c r="G92" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="H92" s="24"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="H92" s="23"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A93" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B93" s="18"/>
-      <c r="C93" s="18"/>
-      <c r="D93" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="E93" s="18"/>
-      <c r="F93" s="18"/>
-      <c r="G93" s="18"/>
-      <c r="H93" s="19"/>
+      <c r="B93" s="19"/>
+      <c r="C93" s="19"/>
+      <c r="D93" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E93" s="19"/>
+      <c r="F93" s="19"/>
+      <c r="G93" s="19"/>
+      <c r="H93" s="20"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A94" s="24"/>
+      <c r="A94" s="25"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
       <c r="D94" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
-      <c r="H94" s="25"/>
+      <c r="H94" s="26"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A95" s="24"/>
+      <c r="A95" s="25"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
       <c r="D95" s="2" t="s">
@@ -7033,106 +7349,106 @@
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
-      <c r="H95" s="25"/>
+      <c r="H95" s="26"/>
     </row>
     <row r="96" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="20"/>
-      <c r="B96" s="22"/>
-      <c r="C96" s="22"/>
-      <c r="D96" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="E96" s="22"/>
-      <c r="F96" s="22"/>
-      <c r="G96" s="22"/>
-      <c r="H96" s="23"/>
+      <c r="A96" s="21"/>
+      <c r="B96" s="23"/>
+      <c r="C96" s="23"/>
+      <c r="D96" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E96" s="23"/>
+      <c r="F96" s="23"/>
+      <c r="G96" s="23"/>
+      <c r="H96" s="24"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A97" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="B97" s="18"/>
-      <c r="C97" s="18"/>
-      <c r="D97" s="18"/>
-      <c r="E97" s="18"/>
-      <c r="F97" s="18"/>
-      <c r="G97" s="54" t="s">
-        <v>60</v>
-      </c>
-      <c r="H97" s="69" t="s">
-        <v>76</v>
+      <c r="A97" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B97" s="19"/>
+      <c r="C97" s="19"/>
+      <c r="D97" s="19"/>
+      <c r="E97" s="19"/>
+      <c r="F97" s="19"/>
+      <c r="G97" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="H97" s="70" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A98" s="24"/>
+      <c r="A98" s="25"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
-      <c r="G98" s="55" t="s">
-        <v>119</v>
-      </c>
-      <c r="H98" s="72" t="s">
-        <v>106</v>
+      <c r="G98" s="56" t="s">
+        <v>118</v>
+      </c>
+      <c r="H98" s="73" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A99" s="24"/>
+      <c r="A99" s="25"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
-      <c r="G99" s="56" t="s">
+      <c r="G99" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="H99" s="72"/>
+      <c r="H99" s="73"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A100" s="24"/>
+      <c r="A100" s="25"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
       <c r="D100" s="1"/>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
-      <c r="G100" s="55" t="s">
-        <v>62</v>
-      </c>
-      <c r="H100" s="72"/>
+      <c r="G100" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="H100" s="73"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A101" s="24"/>
+      <c r="A101" s="25"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
       <c r="D101" s="1"/>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
-      <c r="G101" s="73" t="s">
-        <v>76</v>
-      </c>
-      <c r="H101" s="72"/>
+      <c r="G101" s="74" t="s">
+        <v>75</v>
+      </c>
+      <c r="H101" s="73"/>
     </row>
     <row r="102" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="20"/>
-      <c r="B102" s="22"/>
-      <c r="C102" s="22"/>
-      <c r="D102" s="22"/>
-      <c r="E102" s="22"/>
-      <c r="F102" s="22"/>
-      <c r="G102" s="53" t="s">
-        <v>120</v>
-      </c>
-      <c r="H102" s="70"/>
+      <c r="A102" s="21"/>
+      <c r="B102" s="23"/>
+      <c r="C102" s="23"/>
+      <c r="D102" s="23"/>
+      <c r="E102" s="23"/>
+      <c r="F102" s="23"/>
+      <c r="G102" s="54" t="s">
+        <v>119</v>
+      </c>
+      <c r="H102" s="71"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B103" s="30"/>
-      <c r="C103" s="30"/>
-      <c r="D103" s="30"/>
-      <c r="E103" s="30"/>
-      <c r="F103" s="30"/>
-      <c r="G103" s="30"/>
-      <c r="H103" s="30"/>
+      <c r="B103" s="31"/>
+      <c r="C103" s="31"/>
+      <c r="D103" s="31"/>
+      <c r="E103" s="31"/>
+      <c r="F103" s="31"/>
+      <c r="G103" s="31"/>
+      <c r="H103" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="30">
@@ -7184,36 +7500,36 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>125</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -7320,7 +7636,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B13" s="7">
         <v>0</v>
@@ -7337,7 +7653,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B14" s="7">
         <v>0</v>
@@ -7354,7 +7670,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B15" s="7">
         <v>0</v>
@@ -7371,7 +7687,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="7">
         <v>0</v>
@@ -7388,7 +7704,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
@@ -7405,7 +7721,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B18" s="7">
         <v>0</v>
@@ -7422,7 +7738,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="7">
         <v>0</v>
@@ -7439,7 +7755,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="7">
         <v>0</v>
@@ -7456,7 +7772,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B21" s="7">
         <v>0</v>
@@ -7473,7 +7789,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B22" s="7">
         <v>0</v>
@@ -7490,7 +7806,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B23" s="7">
         <v>0</v>
@@ -7507,7 +7823,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B24" s="7">
         <v>0</v>
@@ -7524,7 +7840,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B25" s="7">
         <v>0</v>
@@ -7541,7 +7857,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B26" s="7">
         <v>0</v>
@@ -7558,7 +7874,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B27" s="7">
         <v>0</v>
@@ -7575,7 +7891,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B28" s="7">
         <v>0</v>
@@ -7592,7 +7908,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B29" s="7">
         <v>0</v>
@@ -7609,7 +7925,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="7">
         <v>0</v>
@@ -7626,7 +7942,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B31" s="7">
         <v>0</v>
@@ -7643,7 +7959,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B32" s="7">
         <v>0</v>
@@ -7660,7 +7976,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B33" s="7">
         <v>0</v>
@@ -7710,40 +8026,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>131</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>133</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -7918,13 +8234,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{405C9297-F11E-4578-88EA-89CDFD73950B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9482BC0-D9A0-4F2E-A662-55F6A6E1E8C5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{495D27A4-2557-4648-A851-BB5BC020AD7E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA586971-1ADE-4638-9DB3-7A0A07ABD948}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5600366F-407E-4B2B-BFE4-5449C85FBAFC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA842A77-17E4-4803-881D-F58312C9A224}"/>
 </file>
</xml_diff>